<commit_message>
Support eight assessment workbook runs
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/ablls-r-template.xlsx
+++ b/public/templates/ablls-r-template.xlsx
@@ -25060,7 +25060,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
@@ -26708,6 +26708,9 @@
       <c r="T24" s="14"/>
       <c r="U24" s="17"/>
       <c r="V24" s="1"/>
+      <c r="AA24" s="38" t="s">
+        <v>10</v>
+      </c>
       <c r="AB24" s="1"/>
       <c r="AH24" s="1"/>
       <c r="AN24" s="1" t="s">
@@ -26730,8 +26733,8 @@
     </row>
     <row r="25" ht="9.0" customHeight="1">
       <c r="A25" s="16"/>
-      <c r="B25" s="80" t="s">
-        <v>85</v>
+      <c r="B25" s="17" t="s">
+        <v>38</v>
       </c>
       <c r="C25" s="80"/>
       <c r="D25" s="81"/>
@@ -26739,13 +26742,14 @@
       <c r="F25" s="80"/>
       <c r="G25" s="80"/>
       <c r="H25" s="80"/>
-      <c r="I25" s="80"/>
+      <c r="I25" s="25" t="s">
+        <v>10</v>
+      </c>
       <c r="J25" s="81"/>
       <c r="K25" s="80"/>
       <c r="L25" s="80"/>
       <c r="M25" s="80"/>
       <c r="N25" s="27"/>
-      <c r="O25" s="23"/>
       <c r="P25" s="1" t="s">
         <v>86</v>
       </c>
@@ -26755,8 +26759,21 @@
       <c r="T25" s="35"/>
       <c r="U25" s="17"/>
       <c r="V25" s="1"/>
+      <c r="AA25" s="76" t="str">
+        <f>I26</f>
+      </c>
       <c r="AB25" s="1"/>
-      <c r="AH25" s="1"/>
+      <c r="AD25" s="51">
+        <f>sum(O26+O89+O148)</f>
+        <v>0</v>
+      </c>
+      <c r="AH25" s="51">
+        <f>(AD25/1484)*100</f>
+        <v>0</v>
+      </c>
+      <c r="AJ25" s="52" t="s">
+        <v>41</v>
+      </c>
       <c r="AN25" s="1" t="s">
         <v>87</v>
       </c>
@@ -26777,22 +26794,23 @@
     </row>
     <row r="26" ht="9.0" customHeight="1">
       <c r="A26" s="16"/>
-      <c r="B26" s="80" t="s">
-        <v>89</v>
-      </c>
+      <c r="B26" s="54"/>
       <c r="C26" s="80"/>
       <c r="D26" s="81"/>
       <c r="E26" s="80"/>
       <c r="F26" s="80"/>
       <c r="G26" s="80"/>
       <c r="H26" s="80"/>
-      <c r="I26" s="80"/>
+      <c r="I26" s="55"/>
       <c r="J26" s="81"/>
       <c r="K26" s="80"/>
       <c r="L26" s="80"/>
       <c r="M26" s="80"/>
       <c r="N26" s="27"/>
-      <c r="O26" s="23"/>
+      <c r="O26" s="59">
+        <f>COUNTIF(E41:H59,7)+countif(K33:N59,7)+countif(Q3:T59,7)+countif(W33:Z59,7)+countif(AC40:AF59,7)+countif(AI31:AL59,7)+countif(AO13:AR59,7)+countif(AU11:AX59,7)+countif(BA51:BD59,7)+O23</f>
+        <v>0</v>
+      </c>
       <c r="P26" s="1" t="s">
         <v>90</v>
       </c>
@@ -26824,8 +26842,8 @@
     </row>
     <row r="27" ht="9.0" customHeight="1">
       <c r="A27" s="16"/>
-      <c r="B27" s="80" t="s">
-        <v>93</v>
+      <c r="B27" s="17" t="s">
+        <v>38</v>
       </c>
       <c r="C27" s="80"/>
       <c r="D27" s="81"/>
@@ -26833,7 +26851,9 @@
       <c r="F27" s="80"/>
       <c r="G27" s="80"/>
       <c r="H27" s="80"/>
-      <c r="I27" s="80"/>
+      <c r="I27" s="25" t="s">
+        <v>10</v>
+      </c>
       <c r="J27" s="81"/>
       <c r="K27" s="80"/>
       <c r="L27" s="80"/>
@@ -26849,6 +26869,9 @@
       <c r="T27" s="35"/>
       <c r="U27" s="17"/>
       <c r="V27" s="1"/>
+      <c r="AA27" s="38" t="s">
+        <v>10</v>
+      </c>
       <c r="AB27" s="1"/>
       <c r="AH27" s="1"/>
       <c r="AN27" s="1" t="s">
@@ -26871,20 +26894,23 @@
     </row>
     <row r="28" ht="9.0" customHeight="1">
       <c r="A28" s="82"/>
-      <c r="B28" s="83"/>
+      <c r="B28" s="54"/>
       <c r="C28" s="83"/>
       <c r="D28" s="84"/>
       <c r="E28" s="83"/>
       <c r="F28" s="83"/>
       <c r="G28" s="83"/>
       <c r="H28" s="83"/>
-      <c r="I28" s="83"/>
+      <c r="I28" s="55"/>
       <c r="J28" s="84"/>
       <c r="K28" s="83"/>
       <c r="L28" s="83"/>
       <c r="M28" s="83"/>
       <c r="N28" s="85"/>
-      <c r="O28" s="86"/>
+      <c r="O28" s="59">
+        <f>COUNTIF(E41:H59,8)+countif(K33:N59,8)+countif(Q3:T59,8)+countif(W33:Z59,8)+countif(AC40:AF59,8)+countif(AI31:AL59,8)+countif(AO13:AR59,8)+countif(AU11:AX59,8)+countif(BA51:BD59,8)+O26</f>
+        <v>0</v>
+      </c>
       <c r="P28" s="1" t="s">
         <v>97</v>
       </c>
@@ -26894,8 +26920,21 @@
       <c r="T28" s="21"/>
       <c r="U28" s="17"/>
       <c r="V28" s="1"/>
+      <c r="AA28" s="76" t="str">
+        <f>I28</f>
+      </c>
       <c r="AB28" s="1"/>
-      <c r="AH28" s="1"/>
+      <c r="AD28" s="51">
+        <f>sum(O28+O92+O151)</f>
+        <v>0</v>
+      </c>
+      <c r="AH28" s="51">
+        <f>(AD28/1484)*100</f>
+        <v>0</v>
+      </c>
+      <c r="AJ28" s="52" t="s">
+        <v>41</v>
+      </c>
       <c r="AN28" s="1" t="s">
         <v>98</v>
       </c>
@@ -30744,13 +30783,20 @@
       <c r="F89" s="80"/>
       <c r="G89" s="80"/>
       <c r="H89" s="80"/>
-      <c r="I89" s="80"/>
+      <c r="I89" s="113" t="str">
+        <f>I26</f>
+      </c>
       <c r="J89" s="81"/>
       <c r="K89" s="80"/>
-      <c r="L89" s="80"/>
+      <c r="L89" s="57">
+        <v>7.0</v>
+      </c>
       <c r="M89" s="80"/>
       <c r="N89" s="27"/>
-      <c r="O89" s="23"/>
+      <c r="O89" s="59">
+        <f>countif(E100:H119,7)+countif(K105:N119,7)+countif(Q86:T119,7)+countif(W108:Z119,7)+countif(AC110:AF119,7)+countif(AI114:AL119,7)+countif(AO103:AR119,7)+countif(AU91:AX119,7)+O86</f>
+        <v>0</v>
+      </c>
       <c r="P89" s="1" t="s">
         <v>406</v>
       </c>
@@ -30931,13 +30977,20 @@
       <c r="F92" s="4"/>
       <c r="G92" s="4"/>
       <c r="H92" s="4"/>
-      <c r="I92" s="4"/>
+      <c r="I92" s="113" t="str">
+        <f>I28</f>
+      </c>
       <c r="J92" s="1"/>
       <c r="K92" s="2"/>
-      <c r="L92" s="2"/>
+      <c r="L92" s="57">
+        <v>8.0</v>
+      </c>
       <c r="M92" s="2"/>
       <c r="N92" s="2"/>
-      <c r="O92" s="4"/>
+      <c r="O92" s="59">
+        <f>countif(E100:H119,8)+countif(K105:N119,8)+countif(Q86:T119,8)+countif(W108:Z119,8)+countif(AC110:AF119,8)+countif(AI114:AL119,8)+countif(AO103:AR119,8)+countif(AU91:AX119,8)+O89</f>
+        <v>0</v>
+      </c>
       <c r="P92" s="1" t="s">
         <v>410</v>
       </c>
@@ -33940,13 +33993,20 @@
       <c r="F148" s="80"/>
       <c r="G148" s="80"/>
       <c r="H148" s="80"/>
-      <c r="I148" s="80"/>
+      <c r="I148" s="113" t="str">
+        <f>I26</f>
+      </c>
       <c r="J148" s="81"/>
       <c r="K148" s="80"/>
-      <c r="L148" s="80"/>
+      <c r="L148" s="57">
+        <v>7.0</v>
+      </c>
       <c r="M148" s="80"/>
       <c r="N148" s="27"/>
-      <c r="O148" s="23"/>
+      <c r="O148" s="59">
+        <f>countif(E171:H180,7)+countif(K174:N180,7)+countif(Q166:T180,7)+countif(W171:Z180,7)+countif(AC174:AF180,7)+countif(AI171:AL180,7)+countif(AO151:AR180,7)+countif(AU153:AX180,7)+O145</f>
+        <v>0</v>
+      </c>
       <c r="P148" s="1"/>
       <c r="V148" s="1"/>
       <c r="AB148" s="1"/>
@@ -34014,11 +34074,20 @@
     </row>
     <row r="151" ht="9.0" customHeight="1">
       <c r="D151" s="1"/>
+      <c r="I151" s="113" t="str">
+        <f>I28</f>
+      </c>
       <c r="J151" s="1"/>
       <c r="K151" s="2"/>
-      <c r="L151" s="2"/>
+      <c r="L151" s="57">
+        <v>8.0</v>
+      </c>
       <c r="M151" s="2"/>
       <c r="N151" s="2"/>
+      <c r="O151" s="59">
+        <f>countif(E171:H180,8)+countif(K174:N180,8)+countif(Q166:T180,8)+countif(W171:Z180,8)+countif(AC174:AF180,8)+countif(AI171:AL180,8)+countif(AO151:AR180,8)+countif(AU153:AX180,8)+O148</f>
+        <v>0</v>
+      </c>
       <c r="P151" s="1"/>
       <c r="V151" s="1"/>
       <c r="AB151" s="1"/>

</xml_diff>